<commit_message>
seats-per-bench max raised from 5 → 6
</commit_message>
<xml_diff>
--- a/backend/format/venue_import.xlsx
+++ b/backend/format/venue_import.xlsx
@@ -645,7 +645,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v xml:space="preserve">  • Venue Name + Type must be unique (no duplicates)</v>
+        <v xml:space="preserve">  • Venue Name + Type must be unique among active venues (archived history may reuse the same name)</v>
       </c>
     </row>
     <row r="25">
@@ -665,7 +665,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v xml:space="preserve">  • Bench Configuration: comma-separated seats per column (2 or 3 only)</v>
+        <v xml:space="preserve">  • Bench Configuration: comma-separated seats per column (1–6 only)</v>
       </c>
     </row>
     <row r="29">

</xml_diff>